<commit_message>
added for quater 1
</commit_message>
<xml_diff>
--- a/data/input/priority_to_train_list.xlsx
+++ b/data/input/priority_to_train_list.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30431"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,15 +10,18 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="127" documentId="8_{65A3C54C-5CDC-4681-A346-798812E8B59A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44B5B01F-D033-463D-92D3-A5DD4B2EFC29}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
     <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -37,21 +40,24 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="67">
   <si>
+    <t>Priority to teach</t>
+  </si>
+  <si>
     <t>Course ID</t>
   </si>
   <si>
     <t>Course Name</t>
   </si>
   <si>
-    <t>Priority to teach</t>
-  </si>
-  <si>
     <t>IGT1IL023</t>
   </si>
   <si>
     <t>Philips Hemo Hospital Engineer</t>
   </si>
   <si>
+    <t>Peter Zandstra</t>
+  </si>
+  <si>
     <t>IGT2IL023</t>
   </si>
   <si>
@@ -70,6 +76,21 @@
     <t>Azurion Essentials - VC007E, FE001, IL006E blend</t>
   </si>
   <si>
+    <t>Christiaan Gelauff</t>
+  </si>
+  <si>
+    <t>Mitchel van Rooij</t>
+  </si>
+  <si>
+    <t>Maurizio Miraglia</t>
+  </si>
+  <si>
+    <t>Tristan de Groot</t>
+  </si>
+  <si>
+    <t>Luis Gonzalez</t>
+  </si>
+  <si>
     <t>IGT2VC005</t>
   </si>
   <si>
@@ -88,18 +109,33 @@
     <t>Interventional Workspot</t>
   </si>
   <si>
+    <t>Junji Noda</t>
+  </si>
+  <si>
+    <t>Chris Spears</t>
+  </si>
+  <si>
     <t>IGT2VC001</t>
   </si>
   <si>
     <t>EchoNavigator</t>
   </si>
   <si>
+    <t>Terry Wiley</t>
+  </si>
+  <si>
     <t>IGT1IL001</t>
   </si>
   <si>
     <t>Allura Xper Release 8.2 Service Training HE</t>
   </si>
   <si>
+    <t>Martienn van Bommel</t>
+  </si>
+  <si>
+    <t>Nick Kuijsten</t>
+  </si>
+  <si>
     <t>IGT1IL003</t>
   </si>
   <si>
@@ -124,12 +160,18 @@
     <t>IGTD Installation &amp; Maintenance</t>
   </si>
   <si>
+    <t>Omar Al Batati</t>
+  </si>
+  <si>
     <t>IGT2IL008</t>
   </si>
   <si>
     <t>BV family R2 - Veradius Essentials</t>
   </si>
   <si>
+    <t>Frank van Mierlo</t>
+  </si>
+  <si>
     <t>IGT2IL009</t>
   </si>
   <si>
@@ -172,6 +214,12 @@
     <t>LumiGuide Foundational Training for Clinical</t>
   </si>
   <si>
+    <t>Corina Nedelea</t>
+  </si>
+  <si>
+    <t>Steven Fokkenrood</t>
+  </si>
+  <si>
     <t>IGT2IL032 (IGT2IL031)</t>
   </si>
   <si>
@@ -182,51 +230,6 @@
   </si>
   <si>
     <t>LumiGuide Introduction for New Hires</t>
-  </si>
-  <si>
-    <t>Peter Zandstra</t>
-  </si>
-  <si>
-    <t>Christiaan Gelauff</t>
-  </si>
-  <si>
-    <t>Mitchel van Rooij</t>
-  </si>
-  <si>
-    <t>Maurizio Miraglia</t>
-  </si>
-  <si>
-    <t>Tristan de Groot</t>
-  </si>
-  <si>
-    <t>Luis Gonzalez</t>
-  </si>
-  <si>
-    <t>Junji Noda</t>
-  </si>
-  <si>
-    <t>Chris Spears</t>
-  </si>
-  <si>
-    <t>Terry Wiley</t>
-  </si>
-  <si>
-    <t>Martienn van Bommel</t>
-  </si>
-  <si>
-    <t>Nick Kuijsten</t>
-  </si>
-  <si>
-    <t>Omar Al Batati</t>
-  </si>
-  <si>
-    <t>Frank van Mierlo</t>
-  </si>
-  <si>
-    <t>Corina Nedelea</t>
-  </si>
-  <si>
-    <t>Steven Fokkenrood</t>
   </si>
   <si>
     <t>Days</t>
@@ -242,7 +245,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -670,7 +673,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -714,17 +717,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1130,30 +1130,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G25"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="7" width="20.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7">
       <c r="A1" s="10"/>
       <c r="B1" s="12"/>
       <c r="C1" s="17" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D1" s="11"/>
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
       <c r="G1" s="12"/>
     </row>
-    <row r="2" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" ht="15.75" thickBot="1">
       <c r="A2" s="13" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C2" s="18">
         <v>1</v>
@@ -1171,7 +1171,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7">
       <c r="A3" s="23" t="s">
         <v>3</v>
       </c>
@@ -1179,176 +1179,176 @@
         <v>4</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="D3" s="8"/>
       <c r="E3" s="8"/>
       <c r="F3" s="8"/>
       <c r="G3" s="9"/>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7">
       <c r="A4" s="25" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="20" t="s">
         <v>5</v>
-      </c>
-      <c r="B4" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="C4" s="20" t="s">
-        <v>49</v>
       </c>
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
       <c r="F4" s="2"/>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7">
       <c r="A5" s="25" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C5" s="20" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
       <c r="G5" s="3"/>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7">
       <c r="A6" s="25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C6" s="20" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>51</v>
+        <v>13</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>53</v>
+        <v>15</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7" s="25" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="C7" s="20" t="s">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="D7" s="2"/>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
       <c r="G7" s="3"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7">
       <c r="A8" s="25" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" s="20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>51</v>
-      </c>
       <c r="G8" s="3"/>
     </row>
-    <row r="9" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" s="1" customFormat="1">
       <c r="A9" s="27" t="s">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="B9" s="28" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C9" s="21" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>56</v>
+        <v>24</v>
       </c>
       <c r="E9" s="4"/>
       <c r="F9" s="4"/>
       <c r="G9" s="5"/>
     </row>
-    <row r="10" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" s="1" customFormat="1">
       <c r="A10" s="27" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B10" s="28" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>55</v>
+        <v>23</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>57</v>
+        <v>27</v>
       </c>
       <c r="E10" s="4"/>
       <c r="F10" s="4"/>
       <c r="G10" s="5"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7">
       <c r="A11" s="25" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="C11" s="20" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
       <c r="G11" s="3"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7">
       <c r="A12" s="25" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="C12" s="20" t="s">
-        <v>58</v>
+        <v>30</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
       <c r="G12" s="3"/>
     </row>
-    <row r="13" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" s="1" customFormat="1">
       <c r="A13" s="27" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="B13" s="28" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="C13" s="21"/>
       <c r="D13" s="4"/>
@@ -1356,12 +1356,12 @@
       <c r="F13" s="4"/>
       <c r="G13" s="5"/>
     </row>
-    <row r="14" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" s="1" customFormat="1">
       <c r="A14" s="27" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B14" s="28" t="s">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="4"/>
@@ -1369,176 +1369,176 @@
       <c r="F14" s="4"/>
       <c r="G14" s="5"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7">
       <c r="A15" s="25" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="C15" s="20" t="s">
-        <v>60</v>
+        <v>40</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
       <c r="G15" s="3"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7">
       <c r="A16" s="25" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="C16" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D16" s="2"/>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
       <c r="G16" s="3"/>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7">
       <c r="A17" s="25" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="C17" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="3"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:7">
       <c r="A18" s="25" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="C18" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D18" s="2"/>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
       <c r="G18" s="3"/>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:7">
       <c r="A19" s="25" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C19" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
       <c r="G19" s="3"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:7">
       <c r="A20" s="25" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="C20" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="3"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7">
       <c r="A21" s="25" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>40</v>
+        <v>53</v>
       </c>
       <c r="C21" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="3"/>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7">
       <c r="A22" s="25" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B22" s="26" t="s">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="C22" s="20" t="s">
-        <v>61</v>
+        <v>43</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="3"/>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7">
       <c r="A23" s="25" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B23" s="26" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="C23" s="20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="3"/>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7">
       <c r="A24" s="25" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B24" s="26" t="s">
-        <v>46</v>
+        <v>61</v>
       </c>
       <c r="C24" s="20" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="3"/>
     </row>
-    <row r="25" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:7" ht="15.75" thickBot="1">
       <c r="A25" s="29" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="B25" s="30" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="C25" s="22" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="D25" s="6" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="6"/>
@@ -1553,7 +1553,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AC22"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="19.7109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="44.85546875" bestFit="1" customWidth="1"/>
@@ -1561,43 +1561,43 @@
     <col min="29" max="29" width="27.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:29" ht="15.75" thickBot="1">
       <c r="A1" s="10"/>
       <c r="B1" s="12"/>
-      <c r="D1" s="37" t="s">
+      <c r="D1" s="42" t="s">
         <v>64</v>
       </c>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
-      <c r="H1" s="37"/>
-      <c r="I1" s="37"/>
-      <c r="J1" s="37"/>
-      <c r="K1" s="37"/>
-      <c r="L1" s="37"/>
-      <c r="M1" s="37"/>
-      <c r="N1" s="37"/>
-      <c r="O1" s="37"/>
-      <c r="P1" s="37"/>
-      <c r="Q1" s="37"/>
-      <c r="R1" s="37"/>
-      <c r="S1" s="37"/>
-      <c r="T1" s="37"/>
-      <c r="U1" s="37"/>
-      <c r="V1" s="37"/>
-      <c r="W1" s="37"/>
-      <c r="X1" s="37"/>
-      <c r="Y1" s="37"/>
-      <c r="Z1" s="37"/>
-      <c r="AA1" s="37"/>
-      <c r="AB1" s="37"/>
-    </row>
-    <row r="2" spans="1:29" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+      <c r="I1" s="42"/>
+      <c r="J1" s="42"/>
+      <c r="K1" s="42"/>
+      <c r="L1" s="42"/>
+      <c r="M1" s="42"/>
+      <c r="N1" s="42"/>
+      <c r="O1" s="42"/>
+      <c r="P1" s="42"/>
+      <c r="Q1" s="42"/>
+      <c r="R1" s="42"/>
+      <c r="S1" s="42"/>
+      <c r="T1" s="42"/>
+      <c r="U1" s="42"/>
+      <c r="V1" s="42"/>
+      <c r="W1" s="42"/>
+      <c r="X1" s="42"/>
+      <c r="Y1" s="42"/>
+      <c r="Z1" s="42"/>
+      <c r="AA1" s="42"/>
+      <c r="AB1" s="42"/>
+    </row>
+    <row r="2" spans="1:29" ht="16.5" thickTop="1" thickBot="1">
       <c r="A2" s="13" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="14" t="s">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D2" s="32">
         <v>1</v>
@@ -1678,26 +1678,26 @@
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29">
       <c r="A3" s="23" t="s">
         <v>3</v>
       </c>
       <c r="B3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="D3" s="38">
+      <c r="D3" s="37">
         <v>3</v>
       </c>
-      <c r="E3" s="39"/>
-      <c r="F3" s="39"/>
+      <c r="E3" s="38"/>
+      <c r="F3" s="38"/>
       <c r="G3" s="2"/>
       <c r="H3" s="3"/>
       <c r="I3" s="35"/>
-      <c r="J3" s="39">
+      <c r="J3" s="38">
         <v>3</v>
       </c>
-      <c r="K3" s="39"/>
-      <c r="L3" s="39"/>
+      <c r="K3" s="38"/>
+      <c r="L3" s="38"/>
       <c r="M3" s="3"/>
       <c r="N3" s="35"/>
       <c r="O3" s="2"/>
@@ -1718,26 +1718,26 @@
         <v>66</v>
       </c>
     </row>
-    <row r="4" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:29">
       <c r="A4" s="25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" s="26" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" s="38">
+        <v>7</v>
+      </c>
+      <c r="D4" s="37">
         <v>3</v>
       </c>
-      <c r="E4" s="39"/>
-      <c r="F4" s="39"/>
+      <c r="E4" s="38"/>
+      <c r="F4" s="38"/>
       <c r="G4" s="2"/>
       <c r="H4" s="3"/>
       <c r="I4" s="35"/>
-      <c r="J4" s="39">
+      <c r="J4" s="38">
         <v>3</v>
       </c>
-      <c r="K4" s="39"/>
-      <c r="L4" s="39"/>
+      <c r="K4" s="38"/>
+      <c r="L4" s="38"/>
       <c r="M4" s="3"/>
       <c r="N4" s="35"/>
       <c r="O4" s="2"/>
@@ -1755,19 +1755,19 @@
       <c r="AA4" s="2"/>
       <c r="AB4" s="3"/>
     </row>
-    <row r="5" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:29">
       <c r="A5" s="25" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B5" s="26" t="s">
-        <v>8</v>
-      </c>
-      <c r="D5" s="38">
+        <v>9</v>
+      </c>
+      <c r="D5" s="37">
         <v>4</v>
       </c>
-      <c r="E5" s="39"/>
-      <c r="F5" s="39"/>
-      <c r="G5" s="39"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
       <c r="H5" s="3"/>
       <c r="I5" s="35"/>
       <c r="J5" s="2"/>
@@ -1790,30 +1790,30 @@
       <c r="AA5" s="2"/>
       <c r="AB5" s="3"/>
     </row>
-    <row r="6" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:29">
       <c r="A6" s="25" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" s="26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="38">
+        <v>11</v>
+      </c>
+      <c r="D6" s="37">
         <v>15</v>
       </c>
-      <c r="E6" s="39"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="39"/>
-      <c r="L6" s="39"/>
-      <c r="M6" s="40"/>
-      <c r="N6" s="38"/>
-      <c r="O6" s="39"/>
-      <c r="P6" s="39"/>
-      <c r="Q6" s="39"/>
-      <c r="R6" s="40"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="39"/>
+      <c r="I6" s="37"/>
+      <c r="J6" s="38"/>
+      <c r="K6" s="38"/>
+      <c r="L6" s="38"/>
+      <c r="M6" s="39"/>
+      <c r="N6" s="37"/>
+      <c r="O6" s="38"/>
+      <c r="P6" s="38"/>
+      <c r="Q6" s="38"/>
+      <c r="R6" s="39"/>
       <c r="S6" s="35"/>
       <c r="T6" s="2"/>
       <c r="U6" s="2"/>
@@ -1825,18 +1825,18 @@
       <c r="AA6" s="2"/>
       <c r="AB6" s="3"/>
     </row>
-    <row r="7" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:29">
       <c r="A7" s="25" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="B7" s="26" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="38">
+        <v>18</v>
+      </c>
+      <c r="D7" s="37">
         <v>3</v>
       </c>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
       <c r="G7" s="2"/>
       <c r="H7" s="3"/>
       <c r="I7" s="35"/>
@@ -1860,18 +1860,18 @@
       <c r="AA7" s="2"/>
       <c r="AB7" s="3"/>
     </row>
-    <row r="8" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:29">
       <c r="A8" s="25" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B8" s="26" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" s="38">
+        <v>20</v>
+      </c>
+      <c r="D8" s="37">
         <v>3</v>
       </c>
-      <c r="E8" s="39"/>
-      <c r="F8" s="39"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
       <c r="G8" s="2"/>
       <c r="H8" s="3"/>
       <c r="I8" s="35"/>
@@ -1895,14 +1895,14 @@
       <c r="AA8" s="2"/>
       <c r="AB8" s="3"/>
     </row>
-    <row r="9" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:29" ht="15.75" thickBot="1">
       <c r="A9" s="25" t="s">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="B9" s="26" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="38">
+        <v>26</v>
+      </c>
+      <c r="D9" s="37">
         <v>1</v>
       </c>
       <c r="E9" s="2"/>
@@ -1910,7 +1910,7 @@
       <c r="G9" s="2"/>
       <c r="H9" s="3"/>
       <c r="I9" s="35"/>
-      <c r="J9" s="41">
+      <c r="J9" s="40">
         <v>1</v>
       </c>
       <c r="K9" s="6"/>
@@ -1918,7 +1918,7 @@
       <c r="M9" s="7"/>
       <c r="N9" s="36"/>
       <c r="O9" s="6"/>
-      <c r="P9" s="41">
+      <c r="P9" s="40">
         <v>1</v>
       </c>
       <c r="Q9" s="6"/>
@@ -1926,47 +1926,47 @@
       <c r="S9" s="36"/>
       <c r="T9" s="6"/>
       <c r="U9" s="6"/>
-      <c r="V9" s="41">
+      <c r="V9" s="40">
         <v>1</v>
       </c>
       <c r="W9" s="7"/>
       <c r="X9" s="36"/>
       <c r="Y9" s="6"/>
       <c r="Z9" s="6"/>
-      <c r="AA9" s="44"/>
-      <c r="AB9" s="42">
+      <c r="AA9" s="6"/>
+      <c r="AB9" s="41">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:29" ht="15.75" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:29" ht="15.75" thickTop="1">
       <c r="A10" s="25" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B10" s="26" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D10" s="35"/>
-      <c r="E10" s="39">
+      <c r="E10" s="38">
         <v>8</v>
       </c>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="40"/>
-      <c r="I10" s="38"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="39"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="38"/>
+      <c r="K10" s="38"/>
+      <c r="L10" s="38"/>
       <c r="M10" s="3"/>
-      <c r="N10" s="38">
+      <c r="N10" s="37">
         <v>8</v>
       </c>
-      <c r="O10" s="39"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="40"/>
-      <c r="S10" s="38"/>
-      <c r="T10" s="39"/>
-      <c r="U10" s="39"/>
+      <c r="O10" s="38"/>
+      <c r="P10" s="38"/>
+      <c r="Q10" s="38"/>
+      <c r="R10" s="39"/>
+      <c r="S10" s="37"/>
+      <c r="T10" s="38"/>
+      <c r="U10" s="38"/>
       <c r="V10" s="2"/>
       <c r="W10" s="3"/>
       <c r="X10" s="35"/>
@@ -1978,35 +1978,35 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:29">
       <c r="A11" s="25" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="B11" s="26" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D11" s="35"/>
-      <c r="E11" s="39">
+      <c r="E11" s="38">
         <v>8</v>
       </c>
-      <c r="F11" s="39"/>
-      <c r="G11" s="39"/>
-      <c r="H11" s="40"/>
-      <c r="I11" s="38"/>
-      <c r="J11" s="39"/>
-      <c r="K11" s="39"/>
-      <c r="L11" s="39"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="39"/>
+      <c r="I11" s="37"/>
+      <c r="J11" s="38"/>
+      <c r="K11" s="38"/>
+      <c r="L11" s="38"/>
       <c r="M11" s="3"/>
-      <c r="N11" s="38">
+      <c r="N11" s="37">
         <v>8</v>
       </c>
-      <c r="O11" s="39"/>
-      <c r="P11" s="39"/>
-      <c r="Q11" s="39"/>
-      <c r="R11" s="40"/>
-      <c r="S11" s="38"/>
-      <c r="T11" s="39"/>
-      <c r="U11" s="39"/>
+      <c r="O11" s="38"/>
+      <c r="P11" s="38"/>
+      <c r="Q11" s="38"/>
+      <c r="R11" s="39"/>
+      <c r="S11" s="37"/>
+      <c r="T11" s="38"/>
+      <c r="U11" s="38"/>
       <c r="V11" s="2"/>
       <c r="W11" s="3"/>
       <c r="X11" s="35"/>
@@ -2018,35 +2018,35 @@
         <v>66</v>
       </c>
     </row>
-    <row r="12" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:29">
       <c r="A12" s="25" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="B12" s="26" t="s">
-        <v>28</v>
+        <v>39</v>
       </c>
       <c r="D12" s="35"/>
-      <c r="E12" s="39">
+      <c r="E12" s="38">
         <v>8</v>
       </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="40"/>
-      <c r="I12" s="38"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="37"/>
+      <c r="J12" s="38"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
       <c r="M12" s="3"/>
-      <c r="N12" s="38">
+      <c r="N12" s="37">
         <v>8</v>
       </c>
-      <c r="O12" s="39"/>
-      <c r="P12" s="39"/>
-      <c r="Q12" s="39"/>
-      <c r="R12" s="40"/>
-      <c r="S12" s="38"/>
-      <c r="T12" s="39"/>
-      <c r="U12" s="39"/>
+      <c r="O12" s="38"/>
+      <c r="P12" s="38"/>
+      <c r="Q12" s="38"/>
+      <c r="R12" s="39"/>
+      <c r="S12" s="37"/>
+      <c r="T12" s="38"/>
+      <c r="U12" s="38"/>
       <c r="V12" s="2"/>
       <c r="W12" s="3"/>
       <c r="X12" s="35"/>
@@ -2058,20 +2058,20 @@
         <v>66</v>
       </c>
     </row>
-    <row r="13" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:29">
       <c r="A13" s="25" t="s">
-        <v>29</v>
+        <v>41</v>
       </c>
       <c r="B13" s="26" t="s">
-        <v>30</v>
-      </c>
-      <c r="D13" s="38">
+        <v>42</v>
+      </c>
+      <c r="D13" s="37">
         <v>5</v>
       </c>
-      <c r="E13" s="39"/>
-      <c r="F13" s="39"/>
-      <c r="G13" s="39"/>
-      <c r="H13" s="40"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="39"/>
       <c r="I13" s="35"/>
       <c r="J13" s="2"/>
       <c r="K13" s="2"/>
@@ -2093,19 +2093,19 @@
       <c r="AA13" s="2"/>
       <c r="AB13" s="3"/>
     </row>
-    <row r="14" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:29">
       <c r="A14" s="25" t="s">
-        <v>31</v>
+        <v>44</v>
       </c>
       <c r="B14" s="26" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="38">
+        <v>45</v>
+      </c>
+      <c r="D14" s="37">
         <v>4</v>
       </c>
-      <c r="E14" s="39"/>
-      <c r="F14" s="39"/>
-      <c r="G14" s="39"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
       <c r="H14" s="3"/>
       <c r="I14" s="35"/>
       <c r="J14" s="2"/>
@@ -2128,19 +2128,19 @@
       <c r="AA14" s="2"/>
       <c r="AB14" s="3"/>
     </row>
-    <row r="15" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:29">
       <c r="A15" s="25" t="s">
-        <v>33</v>
+        <v>46</v>
       </c>
       <c r="B15" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="38">
+        <v>47</v>
+      </c>
+      <c r="D15" s="37">
         <v>4</v>
       </c>
-      <c r="E15" s="39"/>
-      <c r="F15" s="39"/>
-      <c r="G15" s="39"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
       <c r="H15" s="3"/>
       <c r="I15" s="35"/>
       <c r="J15" s="2"/>
@@ -2163,20 +2163,20 @@
       <c r="AA15" s="2"/>
       <c r="AB15" s="3"/>
     </row>
-    <row r="16" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:29">
       <c r="A16" s="25" t="s">
-        <v>35</v>
+        <v>48</v>
       </c>
       <c r="B16" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="D16" s="38">
+        <v>49</v>
+      </c>
+      <c r="D16" s="37">
         <v>5</v>
       </c>
-      <c r="E16" s="39"/>
-      <c r="F16" s="39"/>
-      <c r="G16" s="39"/>
-      <c r="H16" s="40"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="39"/>
       <c r="I16" s="35"/>
       <c r="J16" s="2"/>
       <c r="K16" s="2"/>
@@ -2198,19 +2198,19 @@
       <c r="AA16" s="2"/>
       <c r="AB16" s="3"/>
     </row>
-    <row r="17" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:29">
       <c r="A17" s="25" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="B17" s="26" t="s">
-        <v>38</v>
-      </c>
-      <c r="D17" s="38">
+        <v>51</v>
+      </c>
+      <c r="D17" s="37">
         <v>4</v>
       </c>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="39"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
       <c r="H17" s="3"/>
       <c r="I17" s="35"/>
       <c r="J17" s="2"/>
@@ -2233,20 +2233,20 @@
       <c r="AA17" s="2"/>
       <c r="AB17" s="3"/>
     </row>
-    <row r="18" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:29">
       <c r="A18" s="25" t="s">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="B18" s="26" t="s">
-        <v>40</v>
-      </c>
-      <c r="D18" s="38">
+        <v>53</v>
+      </c>
+      <c r="D18" s="37">
         <v>5</v>
       </c>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="39"/>
-      <c r="H18" s="40"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="39"/>
       <c r="I18" s="35"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -2268,20 +2268,20 @@
       <c r="AA18" s="2"/>
       <c r="AB18" s="3"/>
     </row>
-    <row r="19" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:29">
       <c r="A19" s="25" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="B19" s="26" t="s">
-        <v>42</v>
-      </c>
-      <c r="D19" s="38">
+        <v>55</v>
+      </c>
+      <c r="D19" s="37">
         <v>5</v>
       </c>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="39"/>
-      <c r="H19" s="40"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="39"/>
       <c r="I19" s="35"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -2303,20 +2303,20 @@
       <c r="AA19" s="2"/>
       <c r="AB19" s="3"/>
     </row>
-    <row r="20" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:29">
       <c r="A20" s="25" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B20" s="26" t="s">
-        <v>44</v>
-      </c>
-      <c r="D20" s="45"/>
-      <c r="E20" s="39">
+        <v>57</v>
+      </c>
+      <c r="D20" s="35"/>
+      <c r="E20" s="38">
         <v>4</v>
       </c>
-      <c r="F20" s="39"/>
-      <c r="G20" s="39"/>
-      <c r="H20" s="40"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="39"/>
       <c r="I20" s="35"/>
       <c r="J20" s="2"/>
       <c r="K20" s="2"/>
@@ -2338,20 +2338,20 @@
       <c r="AA20" s="2"/>
       <c r="AB20" s="3"/>
     </row>
-    <row r="21" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:29">
       <c r="A21" s="25" t="s">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="B21" s="26" t="s">
-        <v>46</v>
-      </c>
-      <c r="D21" s="45"/>
-      <c r="E21" s="39">
+        <v>61</v>
+      </c>
+      <c r="D21" s="35"/>
+      <c r="E21" s="38">
         <v>4</v>
       </c>
-      <c r="F21" s="39"/>
-      <c r="G21" s="39"/>
-      <c r="H21" s="40"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="39"/>
       <c r="I21" s="35"/>
       <c r="J21" s="2"/>
       <c r="K21" s="2"/>
@@ -2373,15 +2373,15 @@
       <c r="AA21" s="2"/>
       <c r="AB21" s="3"/>
     </row>
-    <row r="22" spans="1:29" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:29" ht="15.75" thickBot="1">
       <c r="A22" s="29" t="s">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="B22" s="30" t="s">
-        <v>48</v>
+        <v>63</v>
       </c>
       <c r="D22" s="36"/>
-      <c r="E22" s="41">
+      <c r="E22" s="40">
         <v>1</v>
       </c>
       <c r="F22" s="6"/>
@@ -2389,7 +2389,7 @@
       <c r="H22" s="7"/>
       <c r="I22" s="36"/>
       <c r="J22" s="6"/>
-      <c r="K22" s="41">
+      <c r="K22" s="40">
         <v>1</v>
       </c>
       <c r="L22" s="6"/>
@@ -2397,22 +2397,22 @@
       <c r="N22" s="36"/>
       <c r="O22" s="6"/>
       <c r="P22" s="6"/>
-      <c r="Q22" s="41">
+      <c r="Q22" s="40">
         <v>1</v>
       </c>
       <c r="R22" s="7"/>
       <c r="S22" s="36"/>
       <c r="T22" s="6"/>
       <c r="U22" s="6"/>
-      <c r="V22" s="44"/>
-      <c r="W22" s="42">
+      <c r="V22" s="6"/>
+      <c r="W22" s="41">
         <v>1</v>
       </c>
       <c r="X22" s="36"/>
       <c r="Y22" s="6"/>
       <c r="Z22" s="6"/>
       <c r="AA22" s="6"/>
-      <c r="AB22" s="43"/>
+      <c r="AB22" s="7"/>
       <c r="AC22" t="s">
         <v>66</v>
       </c>
@@ -2429,30 +2429,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank workbook (1)","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <TemplafyFormConfiguration><![CDATA[{"formFields":[],"formDataEntries":[]}]]></TemplafyFormConfiguration>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<TemplafyTemplateConfiguration><![CDATA[{"transformationConfigurations":[],"templateName":"Blank workbook (1)","templateDescription":"","enableDocumentContentUpdater":false,"version":"2.0"}]]></TemplafyTemplateConfiguration>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D935B92B-7CB7-4F33-8A9E-9593CFA73A38}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6F80FD2-C12F-42D4-B161-EC42684C5897}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6F80FD2-C12F-42D4-B161-EC42684C5897}">
-  <ds:schemaRefs/>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D935B92B-7CB7-4F33-8A9E-9593CFA73A38}"/>
 </file>
 
 <file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>